<commit_message>
pipeline corrigida mas é preciso corrigir o crawler
</commit_message>
<xml_diff>
--- a/output/resultados.xlsx
+++ b/output/resultados.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -451,16 +451,16 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Captura de ecrã 2026-04-16, às 19.22.57.png</t>
+          <t>Captura de ecrã 2026-04-26, às 11.50.15.png</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>verniz gel cateye meteoro</t>
+          <t>verniz gel agenda cheia</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D2" t="n">
         <v>1</v>
@@ -469,16 +469,16 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Captura de ecrã 2026-04-16, às 19.22.57.png</t>
+          <t>Captura de ecrã 2026-04-26, às 11.50.15.png</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>verniz gel outra vez meias</t>
+          <t>verniz gel a fazer panda</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D3" t="n">
         <v>1</v>
@@ -487,16 +487,16 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Captura de ecrã 2026-04-16, às 19.22.57.png</t>
+          <t>Captura de ecrã 2026-04-26, às 11.50.15.png</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>verniz gel minissaia</t>
+          <t>verniz gel boa luz resolve tudo</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D4" t="n">
         <v>1</v>
@@ -505,16 +505,16 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Captura de ecrã 2026-04-16, às 19.22.57.png</t>
+          <t>Captura de ecrã 2026-04-26, às 11.50.15.png</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>verniz gel natura</t>
+          <t>verniz gel sou basica e depois</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D5" t="n">
         <v>1</v>
@@ -523,16 +523,16 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Captura de ecrã 2026-04-16, às 19.22.57.png</t>
+          <t>Captura de ecrã 2026-04-26, às 11.50.15.png</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>verniz gel terracota</t>
+          <t>verniz gel fingi que nao vi</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D6" t="n">
         <v>1</v>
@@ -541,16 +541,16 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Captura de ecrã 2026-04-16, às 19.22.57.png</t>
+          <t>Captura de ecrã 2026-04-26, às 11.50.15.png</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>verniz gel girassol</t>
+          <t>verniz gel rosa de ultima hora</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D7" t="n">
         <v>1</v>
@@ -559,12 +559,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Captura de ecrã 2026-04-16, às 19.22.57.png</t>
+          <t>Captura de ecrã 2026-04-26, às 11.50.15.png</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>verniz gel sr vinho</t>
+          <t>verniz gel vestido de noiva</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -577,12 +577,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Captura de ecrã 2026-04-16, às 19.22.57.png</t>
+          <t>Captura de ecrã 2026-04-26, às 11.50.15.png</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>top coat milky branco leitoso</t>
+          <t>verniz gel espirito livre</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -595,16 +595,16 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Captura de ecrã 2026-04-16, às 19.22.57.png</t>
+          <t>Captura de ecrã 2026-04-26, às 11.50.15.png</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>tote bag mais cor mais amor</t>
+          <t>verniz gel brigadeiro</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>20</v>
+        <v>3</v>
       </c>
       <c r="D10" t="n">
         <v>1</v>
@@ -613,37 +613,199 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Captura de ecrã 2026-04-16, às 19.22.57.png</t>
+          <t>Captura de ecrã 2026-04-26, às 11.50.15.png</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>verniz gel cateye estrela cadente</t>
+          <t>verniz gel terracota</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D11" t="n">
-        <v>0.9455</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Captura de ecrã 2026-04-16, às 19.22.57.png</t>
+          <t>Captura de ecrã 2026-04-26, às 11.50.15.png</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>verniz gel cateye aurora boreal</t>
+          <t>verniz gel acredita</t>
         </is>
       </c>
       <c r="C12" t="n">
+        <v>3</v>
+      </c>
+      <c r="D12" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Captura de ecrã 2026-04-26, às 11.50.15.png</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>fiber base gel transparente</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>12</v>
+      </c>
+      <c r="D13" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Captura de ecrã 2026-04-26, às 11.50.15.png</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>fiber base gel nude perola</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>6</v>
+      </c>
+      <c r="D14" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Captura de ecrã 2026-04-26, às 11.50.15.png</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>fiber base gel branco leitoso</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>3</v>
+      </c>
+      <c r="D15" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Captura de ecrã 2026-04-26, às 11.50.15.png</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>super primer</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>18</v>
+      </c>
+      <c r="D16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Captura de ecrã 2026-04-26, às 11.50.15.png</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>super top coat</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
         <v>4</v>
       </c>
-      <c r="D12" t="n">
-        <v>0.9254</v>
+      <c r="D17" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Captura de ecrã 2026-04-26, às 11.50.15.png</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>top coat milky nude leitoso</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>6</v>
+      </c>
+      <c r="D18" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Captura de ecrã 2026-04-26, às 11.50.15.png</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>base 5 in 1 repair</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>6</v>
+      </c>
+      <c r="D19" t="n">
+        <v>0.9834000000000001</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Captura de ecrã 2026-04-26, às 11.50.15.png</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>fiber base gel rosa leitoso cintilante</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>8</v>
+      </c>
+      <c r="D20" t="n">
+        <v>0.9754</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Captura de ecrã 2026-04-26, às 11.50.15.png</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>base antes depois</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>4</v>
+      </c>
+      <c r="D21" t="n">
+        <v>0.9532</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
correto no entanto pode ficar ainda melhor
</commit_message>
<xml_diff>
--- a/output/resultados.xlsx
+++ b/output/resultados.xlsx
@@ -451,16 +451,16 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Captura de ecrã 2026-04-26, às 11.50.15.png</t>
+          <t>Captura de ecrã 2026-04-16, às 19.22.57.png</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>verniz gel agenda cheia</t>
+          <t>verniz gel cateye eclipse</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D2" t="n">
         <v>1</v>
@@ -469,16 +469,16 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Captura de ecrã 2026-04-26, às 11.50.15.png</t>
+          <t>Captura de ecrã 2026-04-16, às 19.22.57.png</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>verniz gel a fazer panda</t>
+          <t>verniz gel cateye estrela cadente</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D3" t="n">
         <v>1</v>
@@ -487,16 +487,16 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Captura de ecrã 2026-04-26, às 11.50.15.png</t>
+          <t>Captura de ecrã 2026-04-16, às 19.22.57.png</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>verniz gel boa luz resolve tudo</t>
+          <t>verniz gel cateye nebulosa</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D4" t="n">
         <v>1</v>
@@ -505,16 +505,16 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Captura de ecrã 2026-04-26, às 11.50.15.png</t>
+          <t>Captura de ecrã 2026-04-16, às 19.22.57.png</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>verniz gel sou basica e depois</t>
+          <t>verniz gel cateye meteoro</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D5" t="n">
         <v>1</v>
@@ -523,16 +523,16 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Captura de ecrã 2026-04-26, às 11.50.15.png</t>
+          <t>Captura de ecrã 2026-04-16, às 19.22.57.png</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>verniz gel fingi que nao vi</t>
+          <t>verniz gel cateye cometa</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D6" t="n">
         <v>1</v>
@@ -541,16 +541,16 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Captura de ecrã 2026-04-26, às 11.50.15.png</t>
+          <t>Captura de ecrã 2026-04-16, às 19.22.57.png</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>verniz gel rosa de ultima hora</t>
+          <t>verniz gel cateye aurora boreal</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D7" t="n">
         <v>1</v>
@@ -559,12 +559,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Captura de ecrã 2026-04-26, às 11.50.15.png</t>
+          <t>Captura de ecrã 2026-04-16, às 19.22.57.png</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>verniz gel vestido de noiva</t>
+          <t>verniz gel outra vez meias</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -577,16 +577,16 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Captura de ecrã 2026-04-26, às 11.50.15.png</t>
+          <t>Captura de ecrã 2026-04-16, às 19.22.57.png</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>verniz gel espirito livre</t>
+          <t>verniz gel brigadeiro</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D9" t="n">
         <v>1</v>
@@ -595,12 +595,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Captura de ecrã 2026-04-26, às 11.50.15.png</t>
+          <t>Captura de ecrã 2026-04-16, às 19.22.57.png</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>verniz gel brigadeiro</t>
+          <t>verniz gel caldeirao</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -613,12 +613,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Captura de ecrã 2026-04-26, às 11.50.15.png</t>
+          <t>Captura de ecrã 2026-04-16, às 19.22.57.png</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>verniz gel terracota</t>
+          <t>verniz gel minissaia</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -631,12 +631,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Captura de ecrã 2026-04-26, às 11.50.15.png</t>
+          <t>Captura de ecrã 2026-04-16, às 19.22.57.png</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>verniz gel acredita</t>
+          <t>verniz gel maria moledo</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -649,16 +649,16 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Captura de ecrã 2026-04-26, às 11.50.15.png</t>
+          <t>Captura de ecrã 2026-04-16, às 19.22.57.png</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>fiber base gel transparente</t>
+          <t>verniz gel natura</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="D13" t="n">
         <v>1</v>
@@ -667,16 +667,16 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Captura de ecrã 2026-04-26, às 11.50.15.png</t>
+          <t>Captura de ecrã 2026-04-16, às 19.22.57.png</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>fiber base gel nude perola</t>
+          <t>verniz gel maria creme</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D14" t="n">
         <v>1</v>
@@ -685,12 +685,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Captura de ecrã 2026-04-26, às 11.50.15.png</t>
+          <t>Captura de ecrã 2026-04-16, às 19.22.57.png</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>fiber base gel branco leitoso</t>
+          <t>verniz gel terracota</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -703,16 +703,16 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Captura de ecrã 2026-04-26, às 11.50.15.png</t>
+          <t>Captura de ecrã 2026-04-16, às 19.22.57.png</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>super primer</t>
+          <t>verniz gel girassol</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>18</v>
+        <v>3</v>
       </c>
       <c r="D16" t="n">
         <v>1</v>
@@ -721,16 +721,16 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Captura de ecrã 2026-04-26, às 11.50.15.png</t>
+          <t>Captura de ecrã 2026-04-16, às 19.22.57.png</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>super top coat</t>
+          <t>verniz gel sr vinho</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D17" t="n">
         <v>1</v>
@@ -739,16 +739,16 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Captura de ecrã 2026-04-26, às 11.50.15.png</t>
+          <t>Captura de ecrã 2026-04-16, às 19.22.57.png</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>top coat milky nude leitoso</t>
+          <t>top coat milky branco leitoso</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D18" t="n">
         <v>1</v>
@@ -757,55 +757,55 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Captura de ecrã 2026-04-26, às 11.50.15.png</t>
+          <t>Captura de ecrã 2026-04-16, às 19.22.57.png</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>base 5 in 1 repair</t>
+          <t>imans cateye 5 efeitos</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D19" t="n">
-        <v>0.9834000000000001</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Captura de ecrã 2026-04-26, às 11.50.15.png</t>
+          <t>Captura de ecrã 2026-04-16, às 19.22.57.png</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>fiber base gel rosa leitoso cintilante</t>
+          <t>tote bag mais cor mais amor</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="D20" t="n">
-        <v>0.9754</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Captura de ecrã 2026-04-26, às 11.50.15.png</t>
+          <t>Captura de ecrã 2026-04-16, às 19.22.57.png</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>base antes depois</t>
+          <t>lamp care</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D21" t="n">
-        <v>0.9532</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
problemas resolvidos falta apenas palavras ao contrário
</commit_message>
<xml_diff>
--- a/output/resultados.xlsx
+++ b/output/resultados.xlsx
@@ -417,13 +417,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="55" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="55" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -434,15 +435,20 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Referência</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>Produto</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Quantidade</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Score</t>
         </is>
@@ -451,360 +457,467 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Captura de ecrã 2026-04-16, às 19.22.57.png</t>
+          <t>Captura de ecrã 2026-04-27, às 14.52.48.png</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>91.18.517</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
           <t>verniz gel cateye eclipse</t>
         </is>
       </c>
-      <c r="C2" t="n">
+      <c r="D2" t="n">
         <v>4</v>
       </c>
-      <c r="D2" t="n">
+      <c r="E2" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Captura de ecrã 2026-04-16, às 19.22.57.png</t>
+          <t>Captura de ecrã 2026-04-27, às 14.52.48.png</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
+          <t>91.18.518</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
           <t>verniz gel cateye estrela cadente</t>
         </is>
       </c>
-      <c r="C3" t="n">
+      <c r="D3" t="n">
         <v>4</v>
       </c>
-      <c r="D3" t="n">
+      <c r="E3" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Captura de ecrã 2026-04-16, às 19.22.57.png</t>
+          <t>Captura de ecrã 2026-04-27, às 14.52.48.png</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
+          <t>91.18.519</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
           <t>verniz gel cateye nebulosa</t>
         </is>
       </c>
-      <c r="C4" t="n">
+      <c r="D4" t="n">
         <v>4</v>
       </c>
-      <c r="D4" t="n">
+      <c r="E4" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Captura de ecrã 2026-04-16, às 19.22.57.png</t>
+          <t>Captura de ecrã 2026-04-27, às 14.52.48.png</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
+          <t>91.18.520</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
           <t>verniz gel cateye meteoro</t>
         </is>
       </c>
-      <c r="C5" t="n">
+      <c r="D5" t="n">
         <v>5</v>
       </c>
-      <c r="D5" t="n">
+      <c r="E5" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Captura de ecrã 2026-04-16, às 19.22.57.png</t>
+          <t>Captura de ecrã 2026-04-27, às 14.52.48.png</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
+          <t>91.18.521</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
           <t>verniz gel cateye cometa</t>
         </is>
       </c>
-      <c r="C6" t="n">
+      <c r="D6" t="n">
         <v>4</v>
       </c>
-      <c r="D6" t="n">
+      <c r="E6" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Captura de ecrã 2026-04-16, às 19.22.57.png</t>
+          <t>Captura de ecrã 2026-04-27, às 14.52.48.png</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
+          <t>91.18.522</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
           <t>verniz gel cateye aurora boreal</t>
         </is>
       </c>
-      <c r="C7" t="n">
+      <c r="D7" t="n">
         <v>4</v>
       </c>
-      <c r="D7" t="n">
+      <c r="E7" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Captura de ecrã 2026-04-16, às 19.22.57.png</t>
+          <t>Captura de ecrã 2026-04-27, às 14.52.48.png</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
+          <t>91.18.498</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
           <t>verniz gel outra vez meias</t>
         </is>
       </c>
-      <c r="C8" t="n">
-        <v>3</v>
-      </c>
       <c r="D8" t="n">
+        <v>3</v>
+      </c>
+      <c r="E8" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Captura de ecrã 2026-04-16, às 19.22.57.png</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
+          <t>Captura de ecrã 2026-04-27, às 14.52.48.png</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr"/>
+      <c r="C9" t="inlineStr">
         <is>
           <t>verniz gel brigadeiro</t>
         </is>
       </c>
-      <c r="C9" t="n">
+      <c r="D9" t="n">
         <v>4</v>
       </c>
-      <c r="D9" t="n">
+      <c r="E9" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Captura de ecrã 2026-04-16, às 19.22.57.png</t>
+          <t>Captura de ecrã 2026-04-27, às 14.52.48.png</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
+          <t>91.18.014</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
           <t>verniz gel caldeirao</t>
         </is>
       </c>
-      <c r="C10" t="n">
-        <v>3</v>
-      </c>
       <c r="D10" t="n">
+        <v>3</v>
+      </c>
+      <c r="E10" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Captura de ecrã 2026-04-16, às 19.22.57.png</t>
+          <t>Captura de ecrã 2026-04-27, às 14.52.48.png</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
+          <t>91.18.029</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
           <t>verniz gel minissaia</t>
         </is>
       </c>
-      <c r="C11" t="n">
-        <v>3</v>
-      </c>
       <c r="D11" t="n">
+        <v>3</v>
+      </c>
+      <c r="E11" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Captura de ecrã 2026-04-16, às 19.22.57.png</t>
+          <t>Captura de ecrã 2026-04-27, às 14.52.48.png</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
+          <t>91.18.143</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
           <t>verniz gel maria moledo</t>
         </is>
       </c>
-      <c r="C12" t="n">
-        <v>3</v>
-      </c>
       <c r="D12" t="n">
+        <v>3</v>
+      </c>
+      <c r="E12" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Captura de ecrã 2026-04-16, às 19.22.57.png</t>
+          <t>Captura de ecrã 2026-04-27, às 14.52.48.png</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
+          <t>91.18.088</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
           <t>verniz gel natura</t>
         </is>
       </c>
-      <c r="C13" t="n">
-        <v>3</v>
-      </c>
       <c r="D13" t="n">
+        <v>3</v>
+      </c>
+      <c r="E13" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Captura de ecrã 2026-04-16, às 19.22.57.png</t>
+          <t>Captura de ecrã 2026-04-27, às 14.52.48.png</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
+          <t>91.18.065</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
           <t>verniz gel maria creme</t>
         </is>
       </c>
-      <c r="C14" t="n">
-        <v>3</v>
-      </c>
       <c r="D14" t="n">
+        <v>3</v>
+      </c>
+      <c r="E14" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Captura de ecrã 2026-04-16, às 19.22.57.png</t>
+          <t>Captura de ecrã 2026-04-27, às 14.52.48.png</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
+          <t>91.18.087</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
           <t>verniz gel terracota</t>
         </is>
       </c>
-      <c r="C15" t="n">
-        <v>3</v>
-      </c>
       <c r="D15" t="n">
+        <v>3</v>
+      </c>
+      <c r="E15" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Captura de ecrã 2026-04-16, às 19.22.57.png</t>
+          <t>Captura de ecrã 2026-04-27, às 14.52.48.png</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
+          <t>91.18.380</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
           <t>verniz gel girassol</t>
         </is>
       </c>
-      <c r="C16" t="n">
-        <v>3</v>
-      </c>
       <c r="D16" t="n">
+        <v>3</v>
+      </c>
+      <c r="E16" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Captura de ecrã 2026-04-16, às 19.22.57.png</t>
+          <t>Captura de ecrã 2026-04-27, às 14.52.48.png</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
+          <t>91.18.375</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
           <t>verniz gel sr vinho</t>
         </is>
       </c>
-      <c r="C17" t="n">
-        <v>3</v>
-      </c>
       <c r="D17" t="n">
+        <v>3</v>
+      </c>
+      <c r="E17" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Captura de ecrã 2026-04-16, às 19.22.57.png</t>
+          <t>Captura de ecrã 2026-04-27, às 14.52.48.png</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
+          <t>91.18.330</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
           <t>top coat milky branco leitoso</t>
         </is>
       </c>
-      <c r="C18" t="n">
-        <v>3</v>
-      </c>
       <c r="D18" t="n">
+        <v>3</v>
+      </c>
+      <c r="E18" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Captura de ecrã 2026-04-16, às 19.22.57.png</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
+          <t>Captura de ecrã 2026-04-27, às 14.52.48.png</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr"/>
+      <c r="C19" t="inlineStr">
         <is>
           <t>imans cateye 5 efeitos</t>
         </is>
       </c>
-      <c r="C19" t="n">
+      <c r="D19" t="n">
         <v>8</v>
       </c>
-      <c r="D19" t="n">
+      <c r="E19" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Captura de ecrã 2026-04-16, às 19.22.57.png</t>
+          <t>Captura de ecrã 2026-04-27, às 14.52.48.png</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
+          <t>93.08.016</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
           <t>tote bag mais cor mais amor</t>
         </is>
       </c>
-      <c r="C20" t="n">
-        <v>20</v>
-      </c>
       <c r="D20" t="n">
+        <v>2</v>
+      </c>
+      <c r="E20" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Captura de ecrã 2026-04-16, às 19.22.57.png</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
+          <t>Captura de ecrã 2026-04-27, às 14.52.48.png</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr"/>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>limas pés uso intenso</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>3</v>
+      </c>
+      <c r="E21" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Captura de ecrã 2026-04-27, às 14.52.48.png</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr"/>
+      <c r="C22" t="inlineStr">
         <is>
           <t>lamp care</t>
         </is>
       </c>
-      <c r="C21" t="n">
+      <c r="D22" t="n">
         <v>2</v>
       </c>
-      <c r="D21" t="n">
+      <c r="E22" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
corrigir as unidades dos produtos
</commit_message>
<xml_diff>
--- a/output/resultados.xlsx
+++ b/output/resultados.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -457,21 +457,21 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Captura de ecrã 2026-04-27, às 14.52.48.png</t>
+          <t>Captura de ecrã 2026-04-27, às 14.56.57.png</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>91.18.517</t>
+          <t>91.18.332</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>verniz gel cateye eclipse</t>
+          <t>top coat milky nude leitoso</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E2" t="n">
         <v>1</v>
@@ -480,44 +480,44 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Captura de ecrã 2026-04-27, às 14.52.48.png</t>
+          <t>Captura de ecrã 2026-04-27, às 14.56.57.png</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>91.18.518</t>
+          <t>91.20.044</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>verniz gel cateye estrela cadente</t>
+          <t>creme de maos 500 ml</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E3" t="n">
-        <v>1</v>
+        <v>0.9451000000000001</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Captura de ecrã 2026-04-27, às 14.52.48.png</t>
+          <t>Captura de ecrã 2026-04-27, às 14.56.57.png</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>91.18.519</t>
+          <t>93.01.093</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>verniz gel cateye nebulosa</t>
+          <t>moldes borboleta regular 100</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="E4" t="n">
         <v>1</v>
@@ -526,398 +526,42 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Captura de ecrã 2026-04-27, às 14.52.48.png</t>
+          <t>Captura de ecrã 2026-04-27, às 14.56.57.png</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>91.18.520</t>
+          <t>93.04.001</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>verniz gel cateye meteoro</t>
+          <t>lampada led uv 90</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E5" t="n">
-        <v>1</v>
+        <v>0.982</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Captura de ecrã 2026-04-27, às 14.52.48.png</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>91.18.521</t>
-        </is>
-      </c>
+          <t>Captura de ecrã 2026-04-27, às 14.56.57.png</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr">
         <is>
-          <t>verniz gel cateye cometa</t>
+          <t>lamp care</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E6" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Captura de ecrã 2026-04-27, às 14.52.48.png</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>91.18.522</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>verniz gel cateye aurora boreal</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
-        <v>4</v>
-      </c>
-      <c r="E7" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Captura de ecrã 2026-04-27, às 14.52.48.png</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>91.18.498</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>verniz gel outra vez meias</t>
-        </is>
-      </c>
-      <c r="D8" t="n">
-        <v>3</v>
-      </c>
-      <c r="E8" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Captura de ecrã 2026-04-27, às 14.52.48.png</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr"/>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>verniz gel brigadeiro</t>
-        </is>
-      </c>
-      <c r="D9" t="n">
-        <v>4</v>
-      </c>
-      <c r="E9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Captura de ecrã 2026-04-27, às 14.52.48.png</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>91.18.014</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>verniz gel caldeirao</t>
-        </is>
-      </c>
-      <c r="D10" t="n">
-        <v>3</v>
-      </c>
-      <c r="E10" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Captura de ecrã 2026-04-27, às 14.52.48.png</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>91.18.029</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>verniz gel minissaia</t>
-        </is>
-      </c>
-      <c r="D11" t="n">
-        <v>3</v>
-      </c>
-      <c r="E11" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Captura de ecrã 2026-04-27, às 14.52.48.png</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>91.18.143</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>verniz gel maria moledo</t>
-        </is>
-      </c>
-      <c r="D12" t="n">
-        <v>3</v>
-      </c>
-      <c r="E12" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Captura de ecrã 2026-04-27, às 14.52.48.png</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>91.18.088</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>verniz gel natura</t>
-        </is>
-      </c>
-      <c r="D13" t="n">
-        <v>3</v>
-      </c>
-      <c r="E13" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Captura de ecrã 2026-04-27, às 14.52.48.png</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>91.18.065</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>verniz gel maria creme</t>
-        </is>
-      </c>
-      <c r="D14" t="n">
-        <v>3</v>
-      </c>
-      <c r="E14" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Captura de ecrã 2026-04-27, às 14.52.48.png</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>91.18.087</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>verniz gel terracota</t>
-        </is>
-      </c>
-      <c r="D15" t="n">
-        <v>3</v>
-      </c>
-      <c r="E15" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Captura de ecrã 2026-04-27, às 14.52.48.png</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>91.18.380</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>verniz gel girassol</t>
-        </is>
-      </c>
-      <c r="D16" t="n">
-        <v>3</v>
-      </c>
-      <c r="E16" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Captura de ecrã 2026-04-27, às 14.52.48.png</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>91.18.375</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>verniz gel sr vinho</t>
-        </is>
-      </c>
-      <c r="D17" t="n">
-        <v>3</v>
-      </c>
-      <c r="E17" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Captura de ecrã 2026-04-27, às 14.52.48.png</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>91.18.330</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>top coat milky branco leitoso</t>
-        </is>
-      </c>
-      <c r="D18" t="n">
-        <v>3</v>
-      </c>
-      <c r="E18" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Captura de ecrã 2026-04-27, às 14.52.48.png</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr"/>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>imans cateye 5 efeitos</t>
-        </is>
-      </c>
-      <c r="D19" t="n">
-        <v>8</v>
-      </c>
-      <c r="E19" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Captura de ecrã 2026-04-27, às 14.52.48.png</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>93.08.016</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>tote bag mais cor mais amor</t>
-        </is>
-      </c>
-      <c r="D20" t="n">
-        <v>2</v>
-      </c>
-      <c r="E20" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Captura de ecrã 2026-04-27, às 14.52.48.png</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr"/>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>limas pés uso intenso</t>
-        </is>
-      </c>
-      <c r="D21" t="n">
-        <v>3</v>
-      </c>
-      <c r="E21" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Captura de ecrã 2026-04-27, às 14.52.48.png</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr"/>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>lamp care</t>
-        </is>
-      </c>
-      <c r="D22" t="n">
-        <v>2</v>
-      </c>
-      <c r="E22" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
fine tunnig para os embeddings
</commit_message>
<xml_diff>
--- a/output/resultados.xlsx
+++ b/output/resultados.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -462,19 +462,19 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>91.18.087</t>
+          <t>91.14.060</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>verniz gel terracota</t>
+          <t>box verniz gel sem regras</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E2" t="n">
-        <v>1</v>
+        <v>0.8905</v>
       </c>
     </row>
     <row r="3">
@@ -485,12 +485,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>91.18.364</t>
+          <t>91.18.087</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>verniz gel brigadeiro natura</t>
+          <t>verniz gel terracota</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -508,12 +508,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>91.18.405</t>
+          <t>91.18.364</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>verniz gel moscatel natura</t>
+          <t>verniz gel brigadeiro natura</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -531,12 +531,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>91.18.406</t>
+          <t>91.18.405</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>verniz gel reserva natura</t>
+          <t>verniz gel moscatel natura</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -554,12 +554,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>91.18.407</t>
+          <t>91.18.406</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>verniz gel ruby natura</t>
+          <t>verniz gel reserva natura</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -577,12 +577,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>91.18.408</t>
+          <t>91.18.407</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>verniz gel tawny natura</t>
+          <t>verniz gel ruby natura</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -658,7 +658,7 @@
         <v>3</v>
       </c>
       <c r="E10" t="n">
-        <v>0.9977</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11">
@@ -807,19 +807,19 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>91.18.371</t>
+          <t>81.02.000</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>base solid gel</t>
+          <t>shape gel</t>
         </is>
       </c>
       <c r="D17" t="n">
         <v>6</v>
       </c>
       <c r="E17" t="n">
-        <v>0.9219000000000001</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18">
@@ -842,7 +842,7 @@
         <v>6</v>
       </c>
       <c r="E18" t="n">
-        <v>0.9694</v>
+        <v>1</v>
       </c>
     </row>
     <row r="19">
@@ -980,7 +980,7 @@
         <v>3</v>
       </c>
       <c r="E24" t="n">
-        <v>0.9241</v>
+        <v>1</v>
       </c>
     </row>
     <row r="25">
@@ -1003,7 +1003,7 @@
         <v>10</v>
       </c>
       <c r="E25" t="n">
-        <v>0.9445</v>
+        <v>0.988</v>
       </c>
     </row>
     <row r="26">
@@ -1026,6 +1026,29 @@
         <v>3</v>
       </c>
       <c r="E26" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Captura de ecrã 2026-04-27, às 13.19.55.png</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>93.04.021</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>ultra silence nail drill</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>1</v>
+      </c>
+      <c r="E27" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
a mexer nos alliences
</commit_message>
<xml_diff>
--- a/output/resultados.xlsx
+++ b/output/resultados.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -457,113 +457,109 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Captura de ecrã 2026-04-27, às 13.19.55.png</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>91.14.060</t>
-        </is>
-      </c>
+          <t>Captura de ecrã 2026-04-27, às 20.35.05.png</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr">
         <is>
-          <t>box verniz gel sem regras</t>
+          <t>verniz gel brigadeiro</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>4</v>
+        <v>36</v>
       </c>
       <c r="E2" t="n">
-        <v>0.8905</v>
+        <v>0.88</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Captura de ecrã 2026-04-27, às 13.19.55.png</t>
+          <t>Captura de ecrã 2026-04-27, às 20.35.05.png</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>91.18.087</t>
+          <t>91.18.145</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>verniz gel terracota</t>
+          <t>verniz gel mini bomboca</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>3</v>
+        <v>36</v>
       </c>
       <c r="E3" t="n">
-        <v>1</v>
+        <v>0.9114</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Captura de ecrã 2026-04-27, às 13.19.55.png</t>
+          <t>Captura de ecrã 2026-04-27, às 20.35.05.png</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>91.18.364</t>
+          <t>91.18.269</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>verniz gel brigadeiro natura</t>
+          <t>verniz gel e julieta</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>3</v>
+        <v>36</v>
       </c>
       <c r="E4" t="n">
-        <v>1</v>
+        <v>0.88</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Captura de ecrã 2026-04-27, às 13.19.55.png</t>
+          <t>Captura de ecrã 2026-04-27, às 20.35.05.png</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>91.18.405</t>
+          <t>91.18.033</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>verniz gel moscatel natura</t>
+          <t>verniz gel piquenique</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>3</v>
+        <v>36</v>
       </c>
       <c r="E5" t="n">
-        <v>1</v>
+        <v>0.88</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Captura de ecrã 2026-04-27, às 13.19.55.png</t>
+          <t>Captura de ecrã 2026-04-27, às 20.35.05.png</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>91.18.406</t>
+          <t>91.18.387</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>verniz gel reserva natura</t>
+          <t>base 5 in 1 repair</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>3</v>
+        <v>36</v>
       </c>
       <c r="E6" t="n">
         <v>1</v>
@@ -572,113 +568,113 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Captura de ecrã 2026-04-27, às 13.19.55.png</t>
+          <t>Captura de ecrã 2026-04-27, às 20.35.05.png</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>91.18.407</t>
+          <t>81.04.005</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>verniz gel ruby natura</t>
+          <t>polyacrygel 4 rosa claro</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>3</v>
+        <v>36</v>
       </c>
       <c r="E7" t="n">
-        <v>1</v>
+        <v>0.8782</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Captura de ecrã 2026-04-27, às 13.19.55.png</t>
+          <t>Captura de ecrã 2026-04-27, às 20.35.05.png</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>91.18.422</t>
+          <t>91.20.043</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>verniz gel azul nordico 68</t>
+          <t>creme de maos 50 ml</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>3</v>
+        <v>36</v>
       </c>
       <c r="E8" t="n">
-        <v>1</v>
+        <v>0.88</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Captura de ecrã 2026-04-27, às 13.19.55.png</t>
+          <t>Captura de ecrã 2026-04-27, às 20.35.05.png</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>91.18.484</t>
+          <t>91.12.022</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>verniz gel chama</t>
+          <t>desidrat desidratante de unha</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>3</v>
+        <v>36</v>
       </c>
       <c r="E9" t="n">
-        <v>1</v>
+        <v>0.8905999999999999</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Captura de ecrã 2026-04-27, às 13.19.55.png</t>
+          <t>Captura de ecrã 2026-04-27, às 20.35.05.png</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>91.18.385</t>
+          <t>91.20.051</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>verniz gel hortensia</t>
+          <t>removedor de calosidades e cuticulas 250 ml</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>3</v>
+        <v>36</v>
       </c>
       <c r="E10" t="n">
-        <v>1</v>
+        <v>0.9391</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Captura de ecrã 2026-04-27, às 13.19.55.png</t>
+          <t>Captura de ecrã 2026-04-27, às 20.35.05.png</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>91.18.065</t>
+          <t>93.01.075</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>verniz gel maria creme</t>
+          <t>pincel nail art 000</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>3</v>
+        <v>36</v>
       </c>
       <c r="E11" t="n">
         <v>1</v>
@@ -687,44 +683,44 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Captura de ecrã 2026-04-27, às 13.19.55.png</t>
+          <t>Captura de ecrã 2026-04-27, às 20.35.05.png</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>91.18.194</t>
+          <t>91.20.049</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>verniz gel super mae maria</t>
+          <t>creme de pes 50 ml</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>3</v>
+        <v>36</v>
       </c>
       <c r="E12" t="n">
-        <v>1</v>
+        <v>0.9892</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Captura de ecrã 2026-04-27, às 13.19.55.png</t>
+          <t>Captura de ecrã 2026-04-27, às 20.35.05.png</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>91.18.161</t>
+          <t>91.20.044</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>verniz gel maria rechonchuda</t>
+          <t>creme de maos 500 ml</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>3</v>
+        <v>36</v>
       </c>
       <c r="E13" t="n">
         <v>1</v>
@@ -733,323 +729,24 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Captura de ecrã 2026-04-27, às 13.19.55.png</t>
+          <t>Captura de ecrã 2026-04-27, às 20.35.05.png</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>91.18.183</t>
+          <t>91.20.042</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>verniz gel sardinha</t>
+          <t>esfoliante grao grosso</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>3</v>
+        <v>36</v>
       </c>
       <c r="E14" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Captura de ecrã 2026-04-27, às 13.19.55.png</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>91.18.072</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>super top coat</t>
-        </is>
-      </c>
-      <c r="D15" t="n">
-        <v>6</v>
-      </c>
-      <c r="E15" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Captura de ecrã 2026-04-27, às 13.19.55.png</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>91.18.204</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>top coat gloss</t>
-        </is>
-      </c>
-      <c r="D16" t="n">
-        <v>6</v>
-      </c>
-      <c r="E16" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Captura de ecrã 2026-04-27, às 13.19.55.png</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>81.02.000</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>shape gel</t>
-        </is>
-      </c>
-      <c r="D17" t="n">
-        <v>6</v>
-      </c>
-      <c r="E17" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Captura de ecrã 2026-04-27, às 13.19.55.png</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>91.18.372</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>top coat solid gel</t>
-        </is>
-      </c>
-      <c r="D18" t="n">
-        <v>6</v>
-      </c>
-      <c r="E18" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Captura de ecrã 2026-04-27, às 13.19.55.png</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>91.26.004</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>like gel 104 branco leitoso</t>
-        </is>
-      </c>
-      <c r="D19" t="n">
-        <v>6</v>
-      </c>
-      <c r="E19" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Captura de ecrã 2026-04-27, às 13.19.55.png</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>91.12.012</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>super primer</t>
-        </is>
-      </c>
-      <c r="D20" t="n">
-        <v>6</v>
-      </c>
-      <c r="E20" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Captura de ecrã 2026-04-27, às 13.19.55.png</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>91.18.387</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>base 5 in 1 repair</t>
-        </is>
-      </c>
-      <c r="D21" t="n">
-        <v>6</v>
-      </c>
-      <c r="E21" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Captura de ecrã 2026-04-27, às 13.19.55.png</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>91.18.487</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>base transparente inovita</t>
-        </is>
-      </c>
-      <c r="D22" t="n">
-        <v>3</v>
-      </c>
-      <c r="E22" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Captura de ecrã 2026-04-27, às 13.19.55.png</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>91.18.332</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>top coat milky nude leitoso</t>
-        </is>
-      </c>
-      <c r="D23" t="n">
-        <v>12</v>
-      </c>
-      <c r="E23" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Captura de ecrã 2026-04-27, às 13.19.55.png</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>91.18.504</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>top coat no blue</t>
-        </is>
-      </c>
-      <c r="D24" t="n">
-        <v>3</v>
-      </c>
-      <c r="E24" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>Captura de ecrã 2026-04-27, às 13.19.55.png</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>91.30.001</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>amolecedor de cuticulas</t>
-        </is>
-      </c>
-      <c r="D25" t="n">
-        <v>10</v>
-      </c>
-      <c r="E25" t="n">
-        <v>0.988</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Captura de ecrã 2026-04-27, às 13.19.55.png</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>88.02.001</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>nail liner branco</t>
-        </is>
-      </c>
-      <c r="D26" t="n">
-        <v>3</v>
-      </c>
-      <c r="E26" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>Captura de ecrã 2026-04-27, às 13.19.55.png</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>93.04.021</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>ultra silence nail drill</t>
-        </is>
-      </c>
-      <c r="D27" t="n">
-        <v>1</v>
-      </c>
-      <c r="E27" t="n">
-        <v>1</v>
+        <v>0.8688</v>
       </c>
     </row>
   </sheetData>

</xml_diff>